<commit_message>
feat(results): add new results for scenario_07 with baseline and structured_override configurations
</commit_message>
<xml_diff>
--- a/scenario_07.xlsx
+++ b/scenario_07.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1538,6 +1538,64 @@
         <v>1.8</v>
       </c>
       <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>scenario_07</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>structured_override</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>deepseek-r1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>deepseek-r1-2026-05-03T23:46:20.196068</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>100</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>7</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>473</v>
+      </c>
+      <c r="L19" t="n">
+        <v>4096</v>
+      </c>
+      <c r="M19" t="n">
+        <v>199479</v>
+      </c>
+      <c r="N19" t="n">
+        <v>199479</v>
+      </c>
+      <c r="O19" t="n">
+        <v>199479</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3264,7 +3322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7397,6 +7455,246 @@
       </c>
       <c r="J103" t="n">
         <v>0.9445000000000051</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>scenario_07</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>structured_override</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>deepseek-r1</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>deepseek-r1-2026-05-03T23:46:20.196068</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="n">
+        <v>100</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0.9500000000000055</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>scenario_07</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>structured_override</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>deepseek-r1</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>deepseek-r1-2026-05-03T23:46:20.196068</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>2</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="n">
+        <v>100</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0.9500000000000055</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>scenario_07</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>structured_override</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>deepseek-r1</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>deepseek-r1-2026-05-03T23:46:20.196068</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>3</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="n">
+        <v>100</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0.9500000000000055</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>scenario_07</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>structured_override</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>deepseek-r1</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>deepseek-r1-2026-05-03T23:46:20.196068</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="n">
+        <v>100</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0.9500000000000055</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>scenario_07</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>structured_override</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>deepseek-r1</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>deepseek-r1-2026-05-03T23:46:20.196068</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>5</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="n">
+        <v>100</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0.9500000000000055</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>scenario_07</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>structured_override</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>deepseek-r1</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>deepseek-r1-2026-05-03T23:46:20.196068</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>6</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="n">
+        <v>100</v>
+      </c>
+      <c r="I109" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" t="n">
+        <v>0.9500000000000055</v>
       </c>
     </row>
   </sheetData>

</xml_diff>